<commit_message>
Claim Points Module - Update Claim Product for Automation
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/02_ClaimPoints/ClaimPoints/03_CategoryPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/02_ClaimPoints/ClaimPoints/03_CategoryPageTest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\02_ClaimPoints\ClaimPoints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E95F1F-1C81-4096-8750-027E111554A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF7A3D61-62D3-4C9B-B90B-A2EA8BF87764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="128">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -744,9 +744,6 @@
     <t>Cement</t>
   </si>
   <si>
-    <t>Ambuja Cement</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Verify </t>
     </r>
@@ -1057,25 +1054,6 @@
   </si>
   <si>
     <t>verify_cartdetails_added_categoryname
-cartdetails_clickon_cancelbtn
-cartdetails_clickon_alertbox_yesbtn</t>
-  </si>
-  <si>
-    <t>category_clickon_refreshbtn
-category_selectcategory
-category_selectbrand
-category_enterqty
-hidekeyboard
-category_enter_productremark
-hidekeyboard
-category_clickon_addtocart_btn
-category_enterqty
-hidekeyboard
-category_enter_productremark
-hidekeyboard
-category_clickon_addtocart_btn
-category_clickon_carticon
-verify_cartdetails_productcount
 cartdetails_clickon_cancelbtn
 cartdetails_clickon_alertbox_yesbtn</t>
   </si>
@@ -1114,9 +1092,6 @@
   </si>
   <si>
     <t>verify_cartdetails_qty</t>
-  </si>
-  <si>
-    <t>Ambj001:12,Ambo002:10</t>
   </si>
   <si>
     <t>cartdetails_clickon_cancelbtn
@@ -1212,6 +1187,34 @@
   </si>
   <si>
     <t>10</t>
+  </si>
+  <si>
+    <t>APPIUM Panther</t>
+  </si>
+  <si>
+    <t>APPIUM CEMENT</t>
+  </si>
+  <si>
+    <t>APMCMT0001:12,APMCMT0002:10</t>
+  </si>
+  <si>
+    <t>category_clickon_refreshbtn
+category_selectcategory
+category_selectbrand
+category_enterqty
+hidekeyboard
+category_enter_productremark
+hidekeyboard
+category_clickon_addtocart_btn
+category_enterqty
+hidekeyboard
+category_enter_productremark2
+hidekeyboard
+category_clickon_addtocart_btn
+category_clickon_carticon
+verify_cartdetails_productcount
+cartdetails_clickon_cancelbtn
+cartdetails_clickon_alertbox_yesbtn</t>
   </si>
 </sst>
 </file>
@@ -2174,16 +2177,21 @@
   <dimension ref="A1:N29"/>
   <sheetFormatPr defaultColWidth="12.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="12.1796875" style="2"/>
+    <col min="1" max="1" width="20.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.1796875" style="2"/>
-    <col min="5" max="5" width="50.08984375" style="2" customWidth="1"/>
-    <col min="6" max="7" width="12.1796875" style="2"/>
-    <col min="8" max="8" width="13.81640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="12.1796875" style="2"/>
+    <col min="4" max="4" width="73.08984375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="38.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.6328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.81640625" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.08984375" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="12.1796875" style="2"/>
+    <col min="13" max="13" width="29.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="12.1796875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
@@ -2221,7 +2229,7 @@
         <v>59</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>2</v>
@@ -2466,14 +2474,14 @@
         <v>79</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>71</v>
+        <v>124</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -2497,19 +2505,19 @@
         <v>18</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>5</v>
@@ -2526,21 +2534,21 @@
         <v>19</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
         <v>80</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>81</v>
+        <v>125</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -2560,22 +2568,22 @@
         <v>20</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N12" s="1" t="s">
         <v>5</v>
@@ -2592,10 +2600,10 @@
         <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -2622,28 +2630,28 @@
         <v>22</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>71</v>
+        <v>124</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="N14" s="1" t="s">
         <v>5</v>
@@ -2663,18 +2671,18 @@
         <v>26</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
         <v>80</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>81</v>
+        <v>125</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
@@ -2694,10 +2702,10 @@
         <v>35</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
@@ -2722,10 +2730,10 @@
         <v>36</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
@@ -2753,7 +2761,7 @@
         <v>25</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
@@ -2781,7 +2789,7 @@
         <v>23</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
@@ -2809,13 +2817,13 @@
         <v>24</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
       <c r="I20" s="10" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
       <c r="J20" s="10"/>
       <c r="K20" s="10"/>
@@ -2839,14 +2847,14 @@
         <v>27</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
@@ -2871,7 +2879,7 @@
         <v>28</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
@@ -2901,7 +2909,7 @@
         <v>29</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
@@ -2911,7 +2919,7 @@
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>5</v>
@@ -2931,7 +2939,7 @@
         <v>30</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
@@ -2941,7 +2949,7 @@
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>5</v>
@@ -2958,10 +2966,10 @@
         <v>44</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
@@ -2971,7 +2979,7 @@
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>5</v>
@@ -2991,19 +2999,19 @@
         <v>31</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="N26" s="1" t="s">
         <v>5</v>
@@ -3023,7 +3031,7 @@
         <v>32</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
@@ -3033,7 +3041,7 @@
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>5</v>
@@ -3053,7 +3061,7 @@
         <v>33</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
@@ -3083,19 +3091,19 @@
         <v>49</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="N29" s="1" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Claim Module Logic updated
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/02_ClaimPoints/ClaimPoints/03_CategoryPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/02_ClaimPoints/ClaimPoints/03_CategoryPageTest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\02_ClaimPoints\ClaimPoints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF7A3D61-62D3-4C9B-B90B-A2EA8BF87764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC32FA05-ED7E-483E-BC44-E07F6E4A0CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="127">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -619,9 +619,6 @@
     </r>
   </si>
   <si>
-    <t>Jindal Panther</t>
-  </si>
-  <si>
     <t>roundds</t>
   </si>
   <si>
@@ -689,9 +686,6 @@
     <t>category_enterproductname_insearchfield
 hidekeyboard
 verify_category_productcode_inlist</t>
-  </si>
-  <si>
-    <t>PROD005</t>
   </si>
   <si>
     <r>
@@ -1215,6 +1209,9 @@
 verify_cartdetails_productcount
 cartdetails_clickon_cancelbtn
 cartdetails_clickon_alertbox_yesbtn</t>
+  </si>
+  <si>
+    <t>APMTMT0002</t>
   </si>
 </sst>
 </file>
@@ -2229,7 +2226,7 @@
         <v>59</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>2</v>
@@ -2378,21 +2375,21 @@
         <v>69</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>5</v>
@@ -2412,7 +2409,7 @@
         <v>70</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -2439,22 +2436,22 @@
         <v>16</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>76</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>77</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1" t="s">
-        <v>78</v>
+        <v>126</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>78</v>
+        <v>126</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>5</v>
@@ -2471,17 +2468,17 @@
         <v>17</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -2505,19 +2502,19 @@
         <v>18</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>5</v>
@@ -2534,21 +2531,21 @@
         <v>19</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -2568,22 +2565,22 @@
         <v>20</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="N12" s="1" t="s">
         <v>5</v>
@@ -2600,10 +2597,10 @@
         <v>21</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>95</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>97</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -2613,7 +2610,7 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="N13" s="1" t="s">
         <v>5</v>
@@ -2630,28 +2627,28 @@
         <v>22</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="N14" s="1" t="s">
         <v>5</v>
@@ -2671,18 +2668,18 @@
         <v>26</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
@@ -2702,10 +2699,10 @@
         <v>35</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
@@ -2730,10 +2727,10 @@
         <v>36</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
@@ -2761,7 +2758,7 @@
         <v>25</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
@@ -2789,7 +2786,7 @@
         <v>23</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
@@ -2817,13 +2814,13 @@
         <v>24</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
       <c r="I20" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J20" s="10"/>
       <c r="K20" s="10"/>
@@ -2847,14 +2844,14 @@
         <v>27</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
@@ -2879,7 +2876,7 @@
         <v>28</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
@@ -2909,7 +2906,7 @@
         <v>29</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
@@ -2919,7 +2916,7 @@
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>5</v>
@@ -2939,7 +2936,7 @@
         <v>30</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
@@ -2949,7 +2946,7 @@
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>5</v>
@@ -2966,10 +2963,10 @@
         <v>44</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
@@ -2979,7 +2976,7 @@
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>5</v>
@@ -2999,19 +2996,19 @@
         <v>31</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="N26" s="1" t="s">
         <v>5</v>
@@ -3031,7 +3028,7 @@
         <v>32</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
@@ -3041,7 +3038,7 @@
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>5</v>
@@ -3061,7 +3058,7 @@
         <v>33</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
@@ -3091,19 +3088,19 @@
         <v>49</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="N29" s="1" t="s">
         <v>5</v>

</xml_diff>